<commit_message>
Adiciona lançamento: train malpensa-milan (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,9 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -70,11 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -477,6 +482,31 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>train malpensa-milan</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train Milano Arona (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -507,6 +507,31 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>train Milano Arona</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: marioni cadorna repas guide (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -532,6 +532,31 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>marioni cadorna repas guide</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: marioni cadorna repas guide 5€ (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,31 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>marioni cadorna repas guide</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: golgonda gelati repas guide (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -582,6 +582,31 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>golgonda gelati repas guide</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: to.market (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -607,6 +607,31 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>to.market</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>17.89</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: Faris srl taxe séjour (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -632,6 +632,31 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Faris srl taxe séjour</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: ATM metro milan (19/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -657,6 +657,31 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>ATM metro milan</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: kipoint consigne bagages (20/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -682,6 +682,31 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>kipoint consigne bagages</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: pane tulipane repas guide (20/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -707,6 +707,31 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>pane tulipane repas guide pendant séjour</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: il fornaio (21/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -732,6 +732,31 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>il fornaio</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: filato Carrefour (21/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -757,6 +757,31 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>filato Carrefour</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: Hermitage Sante Caterina (21/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -782,6 +782,31 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Hermitage Sante Caterina</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: billet isola bela+madre + bollo (21/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -807,6 +807,31 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>21/09/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>billet isola bela+madre + bollo</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: il fornaio 2,05€ (22/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -832,6 +832,31 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>il fornaio</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: carrefour (20/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -857,6 +857,31 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>carrefour</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>119.8</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazioni Lenno tremezzo (24/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -882,6 +882,31 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>navigazioni Lenno tremezzo</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazioni orta-san Giulio (22/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -907,6 +907,31 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>navigazioni orta-san Giulio</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: macelleria (24/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -932,6 +932,31 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>macelleria</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: taxi orta (22/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -957,6 +957,31 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>taxi orta</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: cetti (24/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -982,6 +982,31 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>cetti</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>97.06</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: Beretta (23/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1007,6 +1007,31 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Beretta</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: cetti 92,41€ (23/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1032,6 +1032,31 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>cetti</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: villa carlota (24/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1057,6 +1057,31 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>villa carlota</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: crema e cioccolato (24/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1082,6 +1082,31 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>crema e cioccolato</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: Villa melzi (25/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1107,6 +1107,31 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Villa melzi</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: mem pane bellano (25/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1132,6 +1132,31 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>mem pane bellano</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS PIQUE-NIQUES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazioni Lenno bellano (25/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1157,6 +1157,31 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>navigazioni Lenno bellano</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazioni varenna Bellagio (25/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1182,6 +1182,31 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>navigazioni varenna Bellagio</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazioni Bellagio Lenno (25/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1207,6 +1207,31 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>25/09/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>navigazioni Bellagio Lenno</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: navigazione Lenno Côme (26/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1232,6 +1232,31 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>navigazione Lenno Côme</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>184.4</v>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS TRANSPORT DU GROUPE (tickets de bus,…)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: turkeie Kebap déjeuner guide (26/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1257,6 +1257,31 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>turkeie Kebap déjeuner guide</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Adiciona lançamento: train como milan (26/09/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Séjour Lacs Italiens 20-09-26.xlsx
+++ b/planilha/Séjour Lacs Italiens 20-09-26.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1282,6 +1282,31 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>train como milan</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>